<commit_message>
Use the new Đạt Danh logo everywhere
- public/logo-dat-danh.png (from Ref/Đạt Danh_logo_2.png) in header, footer, About
  page, admin login, Open Graph and the Excel quotation header; new file name so the
  image optimiser/CDN cannot keep serving the old THANH DANH artwork
- ĐD mark (public/logo-dat-danh-mark.png) for the favicon and the rotating badge,
  whose ring text now reads SPARE PARTS FACTORY 24H
- Old gear emblem removed; content checklist item ticked

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ayYYJWxMkQ45fCr9uSjrc
</commit_message>
<xml_diff>
--- a/tai-lieu/Bao-gia-Dat-Danh.xlsx
+++ b/tai-lieu/Bao-gia-Dat-Danh.xlsx
@@ -1168,9 +1168,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>542520</xdr:colOff>
+      <xdr:colOff>1161720</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>47160</xdr:rowOff>
+      <xdr:rowOff>9000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1184,7 +1184,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="352440" y="0"/>
-          <a:ext cx="542520" cy="704520"/>
+          <a:ext cx="1161720" cy="666360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Header uses the horizontal Đạt Danh logo; emblem elsewhere
- New public/logo-dat-danh-ngang.png (header) and logo-dat-danh-emblem.png
  (footer, Giới thiệu, admin login, share image, Excel quote header)
- Header back to 80px with non-wrapping nav; compact search on xl

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ayYYJWxMkQ45fCr9uSjrc
</commit_message>
<xml_diff>
--- a/tai-lieu/Bao-gia-Dat-Danh.xlsx
+++ b/tai-lieu/Bao-gia-Dat-Danh.xlsx
@@ -1168,7 +1168,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1161720</xdr:colOff>
+      <xdr:colOff>980640</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>9000</xdr:rowOff>
     </xdr:to>
@@ -1184,7 +1184,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="352440" y="0"/>
-          <a:ext cx="1161720" cy="666360"/>
+          <a:ext cx="980640" cy="666360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1474,7 +1474,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="str">
         <f aca="false">"Số: "&amp;$I$10&amp;"   ·   Ngày: "&amp;TEXT($I$11,"dd/mm/yyyy")</f>
-        <v>Số: BG-2026-001   ·   Ngày: 23/10/2026</v>
+        <v>Số: BG-2026-001   ·   Ngày: 24/10/2026</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="I11" s="11" t="n">
         <f aca="true">TODAY()</f>
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="J11" s="11"/>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="I12" s="11" t="n">
         <f aca="false">I11+15</f>
-        <v>46333</v>
+        <v>46334</v>
       </c>
       <c r="J12" s="11"/>
     </row>

</xml_diff>

<commit_message>
Swap in the final_3 logos (horizontal header + emblem)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ayYYJWxMkQ45fCr9uSjrc
</commit_message>
<xml_diff>
--- a/tai-lieu/Bao-gia-Dat-Danh.xlsx
+++ b/tai-lieu/Bao-gia-Dat-Danh.xlsx
@@ -1168,7 +1168,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>980640</xdr:colOff>
+      <xdr:colOff>1047240</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>9000</xdr:rowOff>
     </xdr:to>
@@ -1184,7 +1184,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="352440" y="0"/>
-          <a:ext cx="980640" cy="666360"/>
+          <a:ext cx="1047240" cy="666360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1474,7 +1474,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="str">
         <f aca="false">"Số: "&amp;$I$10&amp;"   ·   Ngày: "&amp;TEXT($I$11,"dd/mm/yyyy")</f>
-        <v>Số: BG-2026-001   ·   Ngày: 24/10/2026</v>
+        <v>Số: BG-2026-001   ·   Ngày: 27/10/2026</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="I11" s="11" t="n">
         <f aca="true">TODAY()</f>
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="J11" s="11"/>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="I12" s="11" t="n">
         <f aca="false">I11+15</f>
-        <v>46334</v>
+        <v>46337</v>
       </c>
       <c r="J12" s="11"/>
     </row>

</xml_diff>